<commit_message>
feat(F-NAR-019): TREE-DIF-064 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-064.xlsx
+++ b/stories/arbres/TREE-DIF-064.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois de la cabane, un grain de sel brille. Le fil du linge claque, sec, contre le pin. Ça sent la résine chaude, et la mer. Amir vit là, avec papa et maman. La queue rouge tape la marche, impatiente. Tu as vu la queue, Amir ? Elle veut partir ! C'est le cerf-volant, tout rouge. En ce moment, Amir déplie un coin du tissu. Je veux qu'il voie la mer. Il lance trop vite, depuis la marche. Le nez rouge se plie contre le bois. Il ne vole pas ! Le vent va se coucher, tout à l'heure. On prend les affaires, alors ? Merci, tu as dénoué la ficelle.</t>
+          <t>Sur le bois de la cabane, un grain de sel brille. Le fil du linge claque, sec, contre le pin. Ça sent la résine chaude, et la mer. Amir vit là, avec papa et maman. La queue rouge tape la marche, impatiente. Une mouette crie, trop haute pour le rouge. Tu as vu la queue, Amir ? Elle veut partir ! C'est le cerf-volant, tout rouge. En ce moment, Amir déplie un coin du tissu. Je veux qu'il voie la mer. Il lance trop vite, depuis la marche. Le nez rouge se plie contre le bois. Amir souffle, les joues chaudes de dépit. Il ne vole pas ! Le vent va se coucher, tout à l'heure. On prend les affaires, alors ? Merci, tu as dénoué la ficelle.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sur le bois de la cabane, un grain de sel brille. Le fil du linge claque, sec, contre le pin. Ça sent la résine chaude, et la mer. Amir vit là, avec papa et maman. La queue rouge tape la marche, impatiente. Tu as vu la queue, Amir ? Elle veut partir ! C'est le &lt;emphasis level="moderate"&gt;cerf-volant&lt;/emphasis&gt;, tout rouge. En ce moment, Amir déplie un coin du tissu. Je veux qu'il voie la mer. Il lance trop vite, depuis la marche. Le nez rouge se plie contre le bois. Il ne vole pas ! Le vent va se coucher, tout à l'heure. On prend les affaires, alors ? Merci, tu as dénoué la ficelle.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sur le bois de la cabane, un grain de sel brille. Le fil du linge claque, sec, contre le pin. Ça sent la résine chaude, et la mer. Amir vit là, avec papa et maman. La queue rouge tape la marche, impatiente. Une mouette crie, trop haute pour le rouge. Tu as vu la queue, Amir ? Elle veut partir ! C'est le &lt;emphasis level="moderate"&gt;cerf-volant&lt;/emphasis&gt;, tout rouge. En ce moment, Amir déplie un coin du tissu. Je veux qu'il voie la mer. Il lance trop vite, depuis la marche. Le nez rouge se plie contre le bois. Amir souffle, les joues chaudes de dépit. Il ne vole pas ! Le vent va se coucher, tout à l'heure. On prend les affaires, alors ? Merci, tu as dénoué la ficelle.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois de la cabane, un grain de sel brille. Le fil du linge claque, sec, contre le pin. Ça sent la résine chaude, et la mer. Amir vit là, avec papa et maman. La queue rouge tape la marche, impatiente. Tu as vu la queue, Amir ? Elle veut partir ! C'est le &lt;emphasis&gt;cerf-volant&lt;/emphasis&gt;, tout rouge. En ce moment, Amir déplie un coin du tissu. Je veux qu'il voie la mer. Il lance trop vite, depuis la marche. Le nez rouge se plie contre le bois. Il ne vole pas ! Le vent va se coucher, tout à l'heure. On prend les affaires, alors ? Merci, tu as dénoué la ficelle. [pause]</t>
+          <t>Sur le bois de la cabane, un grain de sel brille. Le fil du linge claque, sec, contre le pin. Ça sent la résine chaude, et la mer. Amir vit là, avec papa et maman. La queue rouge tape la marche, impatiente. Une mouette crie, trop haute pour le rouge. Tu as vu la queue, Amir ? Elle veut partir ! C'est le &lt;emphasis&gt;cerf-volant&lt;/emphasis&gt;, tout rouge. En ce moment, Amir déplie un coin du tissu. Je veux qu'il voie la mer. Il lance trop vite, depuis la marche. Le nez rouge se plie contre le bois. Amir souffle, les joues chaudes de dépit. Il ne vole pas ! Le vent va se coucher, tout à l'heure. On prend les affaires, alors ? Merci, tu as dénoué la ficelle. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1346,6 +1346,7 @@
 narrateur|Ça sent la résine chaude, et la mer.
 narrateur|Amir vit là, avec papa et maman.
 narrateur|La queue rouge tape la marche, impatiente.
+narrateur|Une mouette crie, trop haute pour le rouge.
 papa|Tu as vu la queue, Amir ?
 enfant-m|Elle veut partir !
 maman|C'est le cerf-volant, tout rouge.
@@ -1353,6 +1354,7 @@
 enfant-m|Je veux qu'il voie la mer.
 narrateur|Il lance trop vite, depuis la marche.
 narrateur|Le nez rouge se plie contre le bois.
+narrateur|Amir souffle, les joues chaudes de dépit.
 enfant-m|Il ne vole pas !
 papa|Le vent va se coucher, tout à l'heure.
 maman|On prend les affaires, alors ?
@@ -1585,17 +1587,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le tissu rouge, chaud de soleil. Toi, tu vas voir la mer. Il déplie trop vite, et le tissu claque. Tiens le nez, pas la queue. La queue rouge lui fouette le cou. Ta queue me chatouille ! Elle est trop contente. Amir serre les lèvres, puis il ralentit. Maman glisse la ficelle contre son poignet. Le piquet roule contre son genou, lourd. Nez en avant, queue derrière. Le rouge est à toi.</t>
+          <t>Amir prend le tissu rouge, chaud de soleil. Toi, tu vas voir la mer. Il déplie trop vite, et le tissu claque. Tiens le nez, pas la queue. La queue rouge lui fouette le cou. Ta queue me chatouille ! Elle est trop contente. Amir serre les lèvres, puis il ralentit. Le tissu sent le soleil, contre ses paumes. Maman glisse la ficelle contre son poignet. Le piquet roule contre son genou, lourd. Nez en avant, queue derrière. Le rouge est à toi.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir prend le &lt;emphasis level="moderate"&gt;tissu&lt;/emphasis&gt; rouge, chaud de soleil. Toi, tu vas voir la mer. Il déplie trop vite, et le tissu claque. Tiens le nez, pas la queue. La queue rouge lui fouette le cou. Ta queue me chatouille ! Elle est trop contente. Amir serre les lèvres, puis il ralentit. Maman glisse la ficelle contre son poignet. Le piquet roule contre son genou, lourd. Nez en avant, queue derrière. Le rouge est à toi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir prend le &lt;emphasis level="moderate"&gt;tissu&lt;/emphasis&gt; rouge, chaud de soleil. Toi, tu vas voir la mer. Il déplie trop vite, et le tissu claque. Tiens le nez, pas la queue. La queue rouge lui fouette le cou. Ta queue me chatouille ! Elle est trop contente. Amir serre les lèvres, puis il ralentit. Le tissu sent le soleil, contre ses paumes. Maman glisse la ficelle contre son poignet. Le piquet roule contre son genou, lourd. Nez en avant, queue derrière. Le rouge est à toi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le &lt;emphasis&gt;tissu&lt;/emphasis&gt; rouge, chaud de soleil. Toi, tu vas voir la mer. Il déplie trop vite, et le tissu claque. Tiens le nez, pas la queue. La queue rouge lui fouette le cou. Ta queue me chatouille ! Elle est trop contente. Amir serre les lèvres, puis il ralentit. Maman glisse la ficelle contre son poignet. Le piquet roule contre son genou, lourd. Nez en avant, queue derrière. Le rouge est à toi. [pause]</t>
+          <t>Amir prend le &lt;emphasis&gt;tissu&lt;/emphasis&gt; rouge, chaud de soleil. Toi, tu vas voir la mer. Il déplie trop vite, et le tissu claque. Tiens le nez, pas la queue. La queue rouge lui fouette le cou. Ta queue me chatouille ! Elle est trop contente. Amir serre les lèvres, puis il ralentit. Le tissu sent le soleil, contre ses paumes. Maman glisse la ficelle contre son poignet. Le piquet roule contre son genou, lourd. Nez en avant, queue derrière. Le rouge est à toi. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1737,6 +1739,7 @@
 papa|Ta queue me chatouille !
 enfant-m|Elle est trop contente.
 narrateur|Amir serre les lèvres, puis il ralentit.
+narrateur|Le tissu sent le soleil, contre ses paumes.
 narrateur|Maman glisse la ficelle contre son poignet.
 narrateur|Le piquet roule contre son genou, lourd.
 enfant-m|Nez en avant, queue derrière.
@@ -2340,17 +2343,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le tissu rouge est chaud. La crête de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le tissu se tord, trop vite, trop fort. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Entre ses doigts, le tissu rouge est chaud. La crête de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le tissu se tord, trop vite, trop fort. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le tissu rouge est chaud. La &lt;emphasis level="moderate"&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le tissu se tord, trop vite, trop fort. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le tissu rouge est chaud. La &lt;emphasis level="moderate"&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le tissu se tord, trop vite, trop fort. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le tissu rouge est chaud. La &lt;emphasis&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le tissu se tord, trop vite, trop fort. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le tissu rouge est chaud. La &lt;emphasis&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le tissu se tord, trop vite, trop fort. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2495,6 +2498,7 @@
 enfant-m|Il va se déchirer !
 narrateur|La queue claque, trop prise.
 narrateur|Le nez rouge se plie, minuscule.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, le vent est trop grand.
 maman|Le rouge a besoin d'un vent plus petit.
 enfant-m|Alors on fait quoi ?
@@ -2726,17 +2730,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Il baisse le tissu, loin de la crête. Amir descend la pente, les genoux au sable. L'air est plus petit, contre la dune. Il compte un, deux, sans lancer. Un coin du tissu cherche l'air. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, ça tenait mieux.</t>
+          <t>Plus bas, d'abord. Il baisse le tissu, loin de la crête. Amir descend la pente, les genoux au sable. L'air est plus petit, contre la dune. Il compte un, deux, sans lancer. Un coin du tissu cherche l'air. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Il baisse le tissu, loin de la crête. Amir descend la pente, les genoux au sable. L'air est plus petit, contre la dune. Il compte un, deux, sans lancer. Un coin du tissu cherche l'air. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Il baisse le tissu, loin de la crête. Amir descend la pente, les genoux au sable. L'air est plus petit, contre la dune. Il compte un, deux, sans lancer. Un coin du tissu cherche l'air. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Il baisse le tissu, loin de la crête. Amir descend la pente, les genoux au sable. L'air est plus petit, contre la dune. Il compte un, deux, sans lancer. Un coin du tissu cherche l'air. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, ça tenait mieux. [pause]</t>
+          <t>Plus bas, d'abord. Il baisse le tissu, loin de la crête. Amir descend la pente, les genoux au sable. L'air est plus petit, contre la dune. Il compte un, deux, sans lancer. Un coin du tissu cherche l'air. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, ça tenait mieux. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2876,7 +2880,7 @@
 narrateur|L'air est plus petit, contre la dune.
 narrateur|Il compte un, deux, sans lancer.
 narrateur|Un coin du tissu cherche l'air.
-papa|Tu as regardé le vent.
+papa|Ici, le vent est plus petit.
 enfant-m|Ici, tu ne te déchires plus.
 maman|Plus bas, ça tenait mieux.</t>
         </is>
@@ -3095,17 +3099,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>On attend le vent. Il tient le tissu contre lui, sans le lancer. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Le tissu reste plié, sage contre lui. Le vent s'est tu. Le rouge se lève, sans se tordre. Le rouge a eu son silence.</t>
+          <t>On attend le vent. Il tient le tissu contre lui, sans le lancer. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Le tissu reste plié, contre lui. Le vent s'est tu. Le rouge se lève, sans se tordre. Le rouge se tient, sans claquer.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend le vent. Il tient le tissu contre lui, sans le lancer. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Le tissu reste plié, sage contre lui. Le vent s'est tu. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, sans se tordre. Le rouge a eu son silence.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend le vent. Il tient le tissu contre lui, sans le lancer. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Le tissu reste plié, contre lui. Le vent s'est tu. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, sans se tordre. Le rouge se tient, sans claquer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>On attend le vent. Il tient le tissu contre lui, sans le lancer. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Le tissu reste plié, sage contre lui. Le vent s'est tu. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, sans se tordre. Le rouge a eu son silence. [pause]</t>
+          <t>On attend le vent. Il tient le tissu contre lui, sans le lancer. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Le tissu reste plié, contre lui. Le vent s'est tu. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, sans se tordre. Le rouge se tient, sans claquer. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3243,10 +3247,10 @@
 narrateur|Il tient le tissu contre lui, sans le lancer.
 narrateur|Le souffle passe, une fois, puis plus.
 enfant-m|Tu peux partir, maintenant.
-narrateur|Le tissu reste plié, sage contre lui.
+narrateur|Le tissu reste plié, contre lui.
 papa|Le vent s'est tu.
 narrateur|Le rouge se lève, sans se tordre.
-maman|Le rouge a eu son silence.</t>
+maman|Le rouge se tient, sans claquer.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
@@ -3278,17 +3282,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Quand le vent s'est tu, le rouge a vu la mer. On a compté le souffle. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. Le tissu rouge sèche près du seau, un pli salé. Une poussière de sable tourne, puis s'arrête.</t>
+          <t>Quand le vent s'est tu, le rouge a vu la mer. On a compté le souffle. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. Le tissu rouge sèche près du seau, un pli salé. Une poussière de sable tourne, puis s'arrête.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le vent s'est tu, le rouge a vu la mer. On a compté le souffle. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. Le tissu rouge sèche près du seau, un pli salé. Une poussière de sable tourne, puis s'arrête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le vent s'est tu, le rouge a vu la mer. On a compté le souffle. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. Le tissu rouge sèche près du seau, un pli salé. Une poussière de sable tourne, puis s'arrête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le vent s'est tu, le rouge a vu la mer. On a compté le souffle. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. Le tissu rouge sèche près du seau, un pli salé. Une poussière de sable tourne, puis s'arrête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le vent s'est tu, le rouge a vu la mer. On a compté le souffle. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. Le tissu rouge sèche près du seau, un pli salé. Une poussière de sable tourne, puis s'arrête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3424,7 +3428,7 @@
         <is>
           <t>narrateur|Quand le vent s'est tu, le rouge a vu la mer.
 enfant-m|On a compté le souffle.
-papa|Le silence a laissé partir le nez.
+papa|Le nez est parti, sans claquer.
 maman|Rentrez, le pin sent le chaud.
 narrateur|Le tissu rouge sèche près du seau, un pli salé.
 narrateur|Une poussière de sable tourne, puis s'arrête.</t>
@@ -3827,17 +3831,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le tissu rouge est chaud. L'herbe de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Un pli du tissu s'accroche, trop serré. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Entre ses doigts, le tissu rouge est chaud. L'herbe de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Un pli du tissu s'accroche, trop serré. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis level="moderate"&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Un pli du tissu s'accroche, trop serré. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis level="moderate"&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Un pli du tissu s'accroche, trop serré. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Un pli du tissu s'accroche, trop serré. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Un pli du tissu s'accroche, trop serré. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3982,6 +3986,7 @@
 enfant-m|Le fil est coincé !
 narrateur|Une tige tire, puis une autre.
 narrateur|Le rouge n'a plus d'air, trop bas.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, ça s'accroche trop.
 maman|Le fil n'avance plus.
 enfant-m|Alors on fait quoi ?
@@ -4213,17 +4218,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Plus court, d'abord. Il tient le tissu tout près, ficelle courte. L'herbe n'atteint plus le fil. Le rouge se lève, tout petit. Le tissu reste plié un instant, puis s'ouvre. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près.</t>
+          <t>Plus court, d'abord. Il tient le tissu tout près, ficelle courte. L'herbe n'atteint plus le fil. Le rouge se lève, tout petit. Le tissu reste plié un instant, puis s'ouvre. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus court, d'abord. Il tient le tissu tout près, ficelle courte. L'herbe n'atteint plus le fil. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Le tissu reste plié un instant, puis s'ouvre. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus court, d'abord. Il tient le tissu tout près, ficelle courte. L'herbe n'atteint plus le fil. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Le tissu reste plié un instant, puis s'ouvre. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Plus court, d'abord. Il tient le tissu tout près, ficelle courte. L'herbe n'atteint plus le fil. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Le tissu reste plié un instant, puis s'ouvre. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près. [pause]</t>
+          <t>Plus court, d'abord. Il tient le tissu tout près, ficelle courte. L'herbe n'atteint plus le fil. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Le tissu reste plié un instant, puis s'ouvre. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4364,7 +4369,7 @@
 narrateur|Le tissu reste plié un instant, puis s'ouvre.
 maman|Le fil n'a plus accroché.
 enfant-m|Maintenant, tu me vois.
-papa|Tu as commencé tout près.</t>
+papa|Le rouge est parti, tout près.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
@@ -4396,17 +4401,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Tout près, le rouge a repris l'air. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. Le tissu rouge sèche près du seau, un pli salé. Un brin d'herbe se recouche, lent.</t>
+          <t>Tout près, le rouge a repris l'air. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. Le tissu rouge sèche près du seau, un pli salé. Un brin d'herbe se recouche, lent.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout près, le rouge a repris l'air. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. Le tissu rouge sèche près du seau, un pli salé. Un brin d'herbe se recouche, lent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout près, le rouge a repris l'air. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. Le tissu rouge sèche près du seau, un pli salé. Un brin d'herbe se recouche, lent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout près, le rouge a repris l'air. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. Le tissu rouge sèche près du seau, un pli salé. Un brin d'herbe se recouche, lent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout près, le rouge a repris l'air. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. Le tissu rouge sèche près du seau, un pli salé. Un brin d'herbe se recouche, lent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4542,7 +4547,7 @@
         <is>
           <t>narrateur|Tout près, le rouge a repris l'air.
 enfant-m|On a commencé tout court.
-papa|Le silence vous a aidés.
+papa|Les tiges n'ont plus accroché.
 maman|L'herbe sent le sel, moins fort.
 narrateur|Le tissu rouge sèche près du seau, un pli salé.
 narrateur|Un brin d'herbe se recouche, lent.</t>
@@ -4577,17 +4582,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>À genoux, on dénoue. À genoux, il dénoue le tissu, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un coin du tissu cherche l'air. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul.</t>
+          <t>À genoux, on dénoue. À genoux, il dénoue le tissu, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un coin du tissu cherche l'air. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;À genoux, on dénoue. À genoux, il dénoue le tissu, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un coin du tissu cherche l'air. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;À genoux, on dénoue. À genoux, il dénoue le tissu, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un coin du tissu cherche l'air. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>À genoux, on dénoue. À genoux, il dénoue le tissu, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un coin du tissu cherche l'air. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul. [pause]</t>
+          <t>À genoux, on dénoue. À genoux, il dénoue le tissu, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un coin du tissu cherche l'air. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4726,7 +4731,7 @@
 narrateur|Un nœud lâche, puis un autre.
 narrateur|L'herbe se tait, plus loin, toute seule.
 narrateur|Un coin du tissu cherche l'air.
-papa|Tu n'as pas tiré trop fort.
+papa|Le nœud a lâché sans crier.
 enfant-m|C'est pour toi.
 maman|Le nœud a lâché tout seul.</t>
         </is>
@@ -4760,17 +4765,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Quand le nœud s'est tu, le rouge a volé. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. Le tissu rouge sèche près du seau, un pli salé. Un nœud vide reste dans sa paume.</t>
+          <t>Quand le nœud s'est tu, le rouge a volé. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. Le tissu rouge sèche près du seau, un pli salé. Un nœud vide reste dans sa paume.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le nœud s'est tu, le rouge a volé. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. Le tissu rouge sèche près du seau, un pli salé. Un nœud vide reste dans sa paume.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le nœud s'est tu, le rouge a volé. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. Le tissu rouge sèche près du seau, un pli salé. Un nœud vide reste dans sa paume.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le nœud s'est tu, le rouge a volé. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. Le tissu rouge sèche près du seau, un pli salé. Un nœud vide reste dans sa paume.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le nœud s'est tu, le rouge a volé. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. Le tissu rouge sèche près du seau, un pli salé. Un nœud vide reste dans sa paume.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4906,7 +4911,7 @@
         <is>
           <t>narrateur|Quand le nœud s'est tu, le rouge a volé.
 enfant-m|On a dénoué, à genoux.
-papa|Tu n'as pas tiré trop fort.
+papa|Le nœud a lâché sans crier.
 maman|Le fil a parlé tout seul.
 narrateur|Le tissu rouge sèche près du seau, un pli salé.
 narrateur|Un nœud vide reste dans sa paume.</t>
@@ -5305,17 +5310,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le tissu rouge est chaud. L'écume lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le tissu pèse, trop lourd, trop salé. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Entre ses doigts, le tissu rouge est chaud. L'écume lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le tissu pèse, trop lourd, trop salé. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis level="moderate"&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le tissu pèse, trop lourd, trop salé. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis level="moderate"&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le tissu pèse, trop lourd, trop salé. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le tissu pèse, trop lourd, trop salé. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le tissu rouge est chaud. L'&lt;emphasis&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le tissu pèse, trop lourd, trop salé. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5460,8 +5465,9 @@
 enfant-m|Il est tout mouillé !
 narrateur|Une vague revient, trop blanche.
 narrateur|Le rouge n'a plus de vent, trop lourd.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, ça mouille trop.
-maman|Il lui faut du sec, et du temps.
+maman|Le rouge est trop lourd, trop mouillé.
 enfant-m|Alors on fait quoi ?
 papa|Tu vois comment, Amir ?</t>
         </is>
@@ -6059,17 +6065,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>On attend la vague, d'abord. Il tient le tissu, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un coin du tissu cherche l'air. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir.</t>
+          <t>On attend la vague, d'abord. Il tient le tissu, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un coin du tissu cherche l'air. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend la vague, d'abord. Il tient le tissu, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un coin du tissu cherche l'air. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend la vague, d'abord. Il tient le tissu, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un coin du tissu cherche l'air. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>On attend la vague, d'abord. Il tient le tissu, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un coin du tissu cherche l'air. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir. [pause]</t>
+          <t>On attend la vague, d'abord. Il tient le tissu, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un coin du tissu cherche l'air. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6208,9 +6214,9 @@
 narrateur|L'eau va, revient, puis se tait.
 narrateur|Le sable redevient ferme, tout net.
 narrateur|Un coin du tissu cherche l'air.
-papa|Tu n'as pas couru dans l'eau.
+papa|Tes pieds sont restés sur le sable.
 enfant-m|Tu es sec, maintenant.
-maman|Tu as laissé la vague finir.</t>
+maman|La vague a fini toute seule.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
@@ -6242,17 +6248,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Après la vague, le rouge a vu la mer. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. Le tissu rouge sèche près du seau, un pli salé. La vague reste à sa place, plus loin.</t>
+          <t>Après la vague, le rouge a vu la mer. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. Le tissu rouge sèche près du seau, un pli salé. La vague reste à sa place, plus loin.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après la vague, le rouge a vu la mer. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. Le tissu rouge sèche près du seau, un pli salé. La vague reste à sa place, plus loin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après la vague, le rouge a vu la mer. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. Le tissu rouge sèche près du seau, un pli salé. La vague reste à sa place, plus loin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après la vague, le rouge a vu la mer. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. Le tissu rouge sèche près du seau, un pli salé. La vague reste à sa place, plus loin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après la vague, le rouge a vu la mer. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. Le tissu rouge sèche près du seau, un pli salé. La vague reste à sa place, plus loin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6388,7 +6394,7 @@
         <is>
           <t>narrateur|Après la vague, le rouge a vu la mer.
 enfant-m|On a laissé l'eau se taire.
-papa|Tu n'as pas couru dans l'eau.
+papa|Tes pieds sont restés sur le sable.
 maman|Tes doigts sentent le sel.
 narrateur|Le tissu rouge sèche près du seau, un pli salé.
 narrateur|La vague reste à sa place, plus loin.</t>
@@ -6787,17 +6793,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Amir enroule la ficelle autour du poignet. Tu vas tenir le rouge. Il serre trop, et ça marque la peau. Pas trop serré, laisse un peu d'air. Un tour glisse, puis tient. Tu m'as fait un anneau. C'est pour tenir. Papa pose le tissu plié contre le seau. Le piquet reste planté, un peu de travers. Fil, tu restes avec moi. La ficelle est prête.</t>
+          <t>Amir enroule la ficelle autour du poignet. Tu vas tenir le rouge. Il serre trop, et ça marque la peau. Pas trop serré, laisse un peu d'air. Un tour glisse, puis tient. La ficelle sent le sel, un peu collante. Tu m'as fait un anneau. C'est pour tenir. Papa pose le tissu plié contre le seau. Le piquet reste planté, un peu de travers. Fil, tu restes avec moi. La ficelle est prête.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir enroule la &lt;emphasis level="moderate"&gt;ficelle&lt;/emphasis&gt; autour du poignet. Tu vas tenir le rouge. Il serre trop, et ça marque la peau. Pas trop serré, laisse un peu d'air. Un tour glisse, puis tient. Tu m'as fait un anneau. C'est pour tenir. Papa pose le tissu plié contre le seau. Le piquet reste planté, un peu de travers. Fil, tu restes avec moi. La ficelle est prête.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir enroule la &lt;emphasis level="moderate"&gt;ficelle&lt;/emphasis&gt; autour du poignet. Tu vas tenir le rouge. Il serre trop, et ça marque la peau. Pas trop serré, laisse un peu d'air. Un tour glisse, puis tient. La ficelle sent le sel, un peu collante. Tu m'as fait un anneau. C'est pour tenir. Papa pose le tissu plié contre le seau. Le piquet reste planté, un peu de travers. Fil, tu restes avec moi. La ficelle est prête.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Amir enroule la &lt;emphasis&gt;ficelle&lt;/emphasis&gt; autour du poignet. Tu vas tenir le rouge. Il serre trop, et ça marque la peau. Pas trop serré, laisse un peu d'air. Un tour glisse, puis tient. Tu m'as fait un anneau. C'est pour tenir. Papa pose le tissu plié contre le seau. Le piquet reste planté, un peu de travers. Fil, tu restes avec moi. La ficelle est prête. [pause]</t>
+          <t>Amir enroule la &lt;emphasis&gt;ficelle&lt;/emphasis&gt; autour du poignet. Tu vas tenir le rouge. Il serre trop, et ça marque la peau. Pas trop serré, laisse un peu d'air. Un tour glisse, puis tient. La ficelle sent le sel, un peu collante. Tu m'as fait un anneau. C'est pour tenir. Papa pose le tissu plié contre le seau. Le piquet reste planté, un peu de travers. Fil, tu restes avec moi. La ficelle est prête. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6936,6 +6942,7 @@
 narrateur|Il serre trop, et ça marque la peau.
 papa|Pas trop serré, laisse un peu d'air.
 narrateur|Un tour glisse, puis tient.
+narrateur|La ficelle sent le sel, un peu collante.
 maman|Tu m'as fait un anneau.
 enfant-m|C'est pour tenir.
 narrateur|Papa pose le tissu plié contre le seau.
@@ -7541,17 +7548,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Au poignet, la ficelle colle un peu, de sel. La crête de la dune souffle trop fort. Amir lance tout de suite, face au vent. La ficelle siffle, trop tendue, trop vive. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Au poignet, la ficelle colle un peu, de sel. La crête de la dune souffle trop fort. Amir lance tout de suite, face au vent. La ficelle siffle, trop tendue, trop vive. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au poignet, la ficelle colle un peu, de sel. La &lt;emphasis level="moderate"&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. La ficelle siffle, trop tendue, trop vive. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au poignet, la ficelle colle un peu, de sel. La &lt;emphasis level="moderate"&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. La ficelle siffle, trop tendue, trop vive. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Au poignet, la ficelle colle un peu, de sel. La &lt;emphasis&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. La ficelle siffle, trop tendue, trop vive. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Au poignet, la ficelle colle un peu, de sel. La &lt;emphasis&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. La ficelle siffle, trop tendue, trop vive. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7696,6 +7703,7 @@
 enfant-m|Il va se déchirer !
 narrateur|La queue claque, trop prise.
 narrateur|Le nez rouge se plie, minuscule.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, le vent est trop grand.
 maman|Le rouge a besoin d'un vent plus petit.
 enfant-m|Alors on fait quoi ?
@@ -7927,17 +7935,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Il baisse la ficelle, loin de la crête. Amir descend, le fil lâche au poignet. L'air est plus petit, contre la pente. Il compte un, deux, le fil sans siffler. Un bout de ficelle brille, prêt à tenir. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, le fil tenait mieux.</t>
+          <t>Plus bas, d'abord. Il baisse la ficelle, loin de la crête. Amir descend, le fil lâche au poignet. L'air est plus petit, contre la pente. Il compte un, deux, le fil sans siffler. Un bout de ficelle brille, prêt à tenir. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, le fil tenait mieux.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Il baisse la ficelle, loin de la crête. Amir descend, le fil lâche au poignet. L'air est plus petit, contre la pente. Il compte un, deux, le fil sans siffler. Un bout de ficelle brille, prêt à tenir. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, le fil tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Il baisse la ficelle, loin de la crête. Amir descend, le fil lâche au poignet. L'air est plus petit, contre la pente. Il compte un, deux, le fil sans siffler. Un bout de ficelle brille, prêt à tenir. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, le fil tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Il baisse la ficelle, loin de la crête. Amir descend, le fil lâche au poignet. L'air est plus petit, contre la pente. Il compte un, deux, le fil sans siffler. Un bout de ficelle brille, prêt à tenir. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, le fil tenait mieux. [pause]</t>
+          <t>Plus bas, d'abord. Il baisse la ficelle, loin de la crête. Amir descend, le fil lâche au poignet. L'air est plus petit, contre la pente. Il compte un, deux, le fil sans siffler. Un bout de ficelle brille, prêt à tenir. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, le fil tenait mieux. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8077,7 +8085,7 @@
 narrateur|L'air est plus petit, contre la pente.
 narrateur|Il compte un, deux, le fil sans siffler.
 narrateur|Un bout de ficelle brille, prêt à tenir.
-papa|Tu as regardé le vent.
+papa|Ici, le vent est plus petit.
 enfant-m|Ici, tu ne te déchires plus.
 maman|Plus bas, le fil tenait mieux.</t>
         </is>
@@ -8292,17 +8300,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>On attend le vent. Il tient la ficelle, sans la dérouler. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Enroulée, la ficelle attend contre sa manche. Le vent s'est tu. Le rouge se lève, le fil sans crier. Le fil a eu son silence.</t>
+          <t>On attend le vent. Il tient la ficelle, sans la dérouler. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Enroulée, la ficelle attend contre sa manche. Le vent s'est tu. Le rouge se lève, le fil sans crier. Le fil se tient, sans siffler.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend le vent. Il tient la ficelle, sans la dérouler. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Enroulée, la ficelle attend contre sa manche. Le vent s'est tu. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, le fil sans crier. Le fil a eu son silence.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend le vent. Il tient la ficelle, sans la dérouler. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Enroulée, la ficelle attend contre sa manche. Le vent s'est tu. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, le fil sans crier. Le fil se tient, sans siffler.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>On attend le vent. Il tient la ficelle, sans la dérouler. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Enroulée, la ficelle attend contre sa manche. Le vent s'est tu. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, le fil sans crier. Le fil a eu son silence. [pause]</t>
+          <t>On attend le vent. Il tient la ficelle, sans la dérouler. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Enroulée, la ficelle attend contre sa manche. Le vent s'est tu. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, le fil sans crier. Le fil se tient, sans siffler. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8443,7 +8451,7 @@
 narrateur|Enroulée, la ficelle attend contre sa manche.
 papa|Le vent s'est tu.
 narrateur|Le rouge se lève, le fil sans crier.
-maman|Le fil a eu son silence.</t>
+maman|Le fil se tient, sans siffler.</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr">
@@ -8475,17 +8483,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Quand le vent s'est tu, le fil a laissé le rouge. On a compté, le fil sans siffler. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. La ficelle reste enroulée, un bout collant de sel. Le fil ne siffle plus, et le rouge tient.</t>
+          <t>Quand le vent s'est tu, le fil a laissé le rouge. On a compté, le fil sans siffler. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. La ficelle reste enroulée, un bout collant de sel. Le fil ne siffle plus, et le rouge tient.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le vent s'est tu, le fil a laissé le rouge. On a compté, le fil sans siffler. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. La ficelle reste enroulée, un bout collant de sel. Le fil ne siffle plus, et le rouge tient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le vent s'est tu, le fil a laissé le rouge. On a compté, le fil sans siffler. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. La ficelle reste enroulée, un bout collant de sel. Le fil ne siffle plus, et le rouge tient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le vent s'est tu, le fil a laissé le rouge. On a compté, le fil sans siffler. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. La ficelle reste enroulée, un bout collant de sel. Le fil ne siffle plus, et le rouge tient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le vent s'est tu, le fil a laissé le rouge. On a compté, le fil sans siffler. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. La ficelle reste enroulée, un bout collant de sel. Le fil ne siffle plus, et le rouge tient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8621,7 +8629,7 @@
         <is>
           <t>narrateur|Quand le vent s'est tu, le fil a laissé le rouge.
 enfant-m|On a compté, le fil sans siffler.
-papa|Le silence a laissé partir le nez.
+papa|Le nez est parti, sans claquer.
 maman|Rentrez, le pin sent le chaud.
 narrateur|La ficelle reste enroulée, un bout collant de sel.
 narrateur|Le fil ne siffle plus, et le rouge tient.</t>
@@ -9020,17 +9028,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Au poignet, la ficelle colle un peu, de sel. L'herbe de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. La ficelle fait un nœud, trop vite. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Au poignet, la ficelle colle un peu, de sel. L'herbe de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. La ficelle fait un nœud, trop vite. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis level="moderate"&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. La ficelle fait un nœud, trop vite. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis level="moderate"&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. La ficelle fait un nœud, trop vite. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. La ficelle fait un nœud, trop vite. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. La ficelle fait un nœud, trop vite. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9175,6 +9183,7 @@
 enfant-m|Le fil est coincé !
 narrateur|Une tige tire, puis une autre.
 narrateur|Le rouge n'a plus d'air, trop bas.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, ça s'accroche trop.
 maman|Le fil n'avance plus.
 enfant-m|Alors on fait quoi ?
@@ -9406,17 +9415,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Plus court, d'abord. Il déroule peu de ficelle, tout court. L'herbe n'atteint plus le fil. Le rouge se lève, tout petit. Enroulée, la ficelle reste sage un instant. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près.</t>
+          <t>Plus court, d'abord. Il déroule peu de ficelle, tout court. L'herbe n'atteint plus le fil. Le rouge se lève, tout petit. Enroulée, la ficelle reste sage un instant. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus court, d'abord. Il déroule peu de ficelle, tout court. L'herbe n'atteint plus le fil. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Enroulée, la ficelle reste sage un instant. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus court, d'abord. Il déroule peu de ficelle, tout court. L'herbe n'atteint plus le fil. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Enroulée, la ficelle reste sage un instant. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Plus court, d'abord. Il déroule peu de ficelle, tout court. L'herbe n'atteint plus le fil. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Enroulée, la ficelle reste sage un instant. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près. [pause]</t>
+          <t>Plus court, d'abord. Il déroule peu de ficelle, tout court. L'herbe n'atteint plus le fil. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Enroulée, la ficelle reste sage un instant. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9557,7 +9566,7 @@
 narrateur|Enroulée, la ficelle reste sage un instant.
 maman|Le fil n'a plus accroché.
 enfant-m|Maintenant, tu me vois.
-papa|Tu as commencé tout près.</t>
+papa|Le rouge est parti, tout près.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr">
@@ -9589,17 +9598,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Tout près, le fil court, net, au-dessus des tiges. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. La ficelle reste enroulée, un bout collant de sel. Le fil court, net, au-dessus des tiges.</t>
+          <t>Tout près, le fil court, net, au-dessus des tiges. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. La ficelle reste enroulée, un bout collant de sel. Le fil court, net, au-dessus des tiges.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout près, le fil court, net, au-dessus des tiges. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. La ficelle reste enroulée, un bout collant de sel. Le fil court, net, au-dessus des tiges.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout près, le fil court, net, au-dessus des tiges. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. La ficelle reste enroulée, un bout collant de sel. Le fil court, net, au-dessus des tiges.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout près, le fil court, net, au-dessus des tiges. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. La ficelle reste enroulée, un bout collant de sel. Le fil court, net, au-dessus des tiges.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout près, le fil court, net, au-dessus des tiges. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. La ficelle reste enroulée, un bout collant de sel. Le fil court, net, au-dessus des tiges.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9735,7 +9744,7 @@
         <is>
           <t>narrateur|Tout près, le fil court, net, au-dessus des tiges.
 enfant-m|On a commencé tout court.
-papa|Le silence vous a aidés.
+papa|Les tiges n'ont plus accroché.
 maman|L'herbe sent le sel, moins fort.
 narrateur|La ficelle reste enroulée, un bout collant de sel.
 narrateur|Le fil court, net, au-dessus des tiges.</t>
@@ -9770,17 +9779,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>À genoux, on dénoue. À genoux, il dénoue la ficelle, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un bout de ficelle brille, prêt à tenir. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul.</t>
+          <t>À genoux, on dénoue. À genoux, il dénoue la ficelle, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un bout de ficelle brille, prêt à tenir. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;À genoux, on dénoue. À genoux, il dénoue la ficelle, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un bout de ficelle brille, prêt à tenir. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;À genoux, on dénoue. À genoux, il dénoue la ficelle, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un bout de ficelle brille, prêt à tenir. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>À genoux, on dénoue. À genoux, il dénoue la ficelle, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un bout de ficelle brille, prêt à tenir. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul. [pause]</t>
+          <t>À genoux, on dénoue. À genoux, il dénoue la ficelle, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. Un bout de ficelle brille, prêt à tenir. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9919,7 +9928,7 @@
 narrateur|Un nœud lâche, puis un autre.
 narrateur|L'herbe se tait, plus loin, toute seule.
 narrateur|Un bout de ficelle brille, prêt à tenir.
-papa|Tu n'as pas tiré trop fort.
+papa|Le nœud a lâché sans crier.
 enfant-m|C'est pour toi.
 maman|Le nœud a lâché tout seul.</t>
         </is>
@@ -9953,17 +9962,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Quand le nœud s'est tu, le fil a parlé. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. La ficelle reste enroulée, un bout collant de sel. Un tour de ficelle s'endort contre sa manche.</t>
+          <t>Quand le nœud s'est tu, le fil a parlé. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. La ficelle reste enroulée, un bout collant de sel. Un tour de ficelle s'endort contre sa manche.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le nœud s'est tu, le fil a parlé. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. La ficelle reste enroulée, un bout collant de sel. Un tour de ficelle s'endort contre sa manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le nœud s'est tu, le fil a parlé. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. La ficelle reste enroulée, un bout collant de sel. Un tour de ficelle s'endort contre sa manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le nœud s'est tu, le fil a parlé. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. La ficelle reste enroulée, un bout collant de sel. Un tour de ficelle s'endort contre sa manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le nœud s'est tu, le fil a parlé. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. La ficelle reste enroulée, un bout collant de sel. Un tour de ficelle s'endort contre sa manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10099,7 +10108,7 @@
         <is>
           <t>narrateur|Quand le nœud s'est tu, le fil a parlé.
 enfant-m|On a dénoué, à genoux.
-papa|Tu n'as pas tiré trop fort.
+papa|Le nœud a lâché sans crier.
 maman|Le fil a parlé tout seul.
 narrateur|La ficelle reste enroulée, un bout collant de sel.
 narrateur|Un tour de ficelle s'endort contre sa manche.</t>
@@ -10498,17 +10507,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Au poignet, la ficelle colle un peu, de sel. L'écume lèche le sable, trop près. Amir avance trop près, et une vague lèche. La ficelle goutte, trop mouillée, trop froide. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Au poignet, la ficelle colle un peu, de sel. L'écume lèche le sable, trop près. Amir avance trop près, et une vague lèche. La ficelle goutte, trop mouillée, trop froide. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis level="moderate"&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. La ficelle goutte, trop mouillée, trop froide. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis level="moderate"&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. La ficelle goutte, trop mouillée, trop froide. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. La ficelle goutte, trop mouillée, trop froide. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Au poignet, la ficelle colle un peu, de sel. L'&lt;emphasis&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. La ficelle goutte, trop mouillée, trop froide. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10653,8 +10662,9 @@
 enfant-m|Il est tout mouillé !
 narrateur|Une vague revient, trop blanche.
 narrateur|Le rouge n'a plus de vent, trop lourd.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, ça mouille trop.
-maman|Il lui faut du sec, et du temps.
+maman|Le rouge est trop lourd, trop mouillé.
 enfant-m|Alors on fait quoi ?
 papa|Tu vois comment, Amir ?</t>
         </is>
@@ -11248,17 +11258,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>On attend la vague, d'abord. Il tient la ficelle, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un bout de ficelle brille, prêt à tenir. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir.</t>
+          <t>On attend la vague, d'abord. Il tient la ficelle, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un bout de ficelle brille, prêt à tenir. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend la vague, d'abord. Il tient la ficelle, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un bout de ficelle brille, prêt à tenir. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend la vague, d'abord. Il tient la ficelle, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un bout de ficelle brille, prêt à tenir. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>On attend la vague, d'abord. Il tient la ficelle, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un bout de ficelle brille, prêt à tenir. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir. [pause]</t>
+          <t>On attend la vague, d'abord. Il tient la ficelle, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. Un bout de ficelle brille, prêt à tenir. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11397,9 +11407,9 @@
 narrateur|L'eau va, revient, puis se tait.
 narrateur|Le sable redevient ferme, tout net.
 narrateur|Un bout de ficelle brille, prêt à tenir.
-papa|Tu n'as pas couru dans l'eau.
+papa|Tes pieds sont restés sur le sable.
 enfant-m|Tu es sec, maintenant.
-maman|Tu as laissé la vague finir.</t>
+maman|La vague a fini toute seule.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr">
@@ -11431,17 +11441,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Après la vague, le fil a vu la mer, sec. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. La ficelle reste enroulée, un bout collant de sel. Un bout collant de sel sèche au poignet.</t>
+          <t>Après la vague, le fil a vu la mer, sec. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. La ficelle reste enroulée, un bout collant de sel. Un bout collant de sel sèche au poignet.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après la vague, le fil a vu la mer, sec. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. La ficelle reste enroulée, un bout collant de sel. Un bout collant de sel sèche au poignet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après la vague, le fil a vu la mer, sec. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. La ficelle reste enroulée, un bout collant de sel. Un bout collant de sel sèche au poignet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après la vague, le fil a vu la mer, sec. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. La ficelle reste enroulée, un bout collant de sel. Un bout collant de sel sèche au poignet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après la vague, le fil a vu la mer, sec. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. La ficelle reste enroulée, un bout collant de sel. Un bout collant de sel sèche au poignet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11577,7 +11587,7 @@
         <is>
           <t>narrateur|Après la vague, le fil a vu la mer, sec.
 enfant-m|On a laissé l'eau se taire.
-papa|Tu n'as pas couru dans l'eau.
+papa|Tes pieds sont restés sur le sable.
 maman|Tes doigts sentent le sel.
 narrateur|La ficelle reste enroulée, un bout collant de sel.
 narrateur|Un bout collant de sel sèche au poignet.</t>
@@ -11976,17 +11986,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Amir lève le piquet, le bois chaud. Tu vas tenir le fil. Il plante trop fort, et le bois penche. Pointe vers le bas, sans forcer. Le bois tape le sable, un toc. Il a tracé une ligne, comme un serpent. C'est le chemin. Maman glisse le tissu sous son autre bras. La ficelle pend contre sa manche. Piquet, je te porte. Le piquet est prêt, on avance.</t>
+          <t>Amir lève le piquet, le bois chaud. Tu vas tenir le fil. Il plante trop fort, et le bois penche. Pointe vers le bas, sans forcer. Le bois tape le sable, un toc. Amir essuie le sable sur sa paume. Il a tracé une ligne, comme un serpent. C'est le chemin. Maman glisse le tissu sous son autre bras. La ficelle pend contre sa manche. Piquet, je te porte. Le piquet est prêt, on avance.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir lève le &lt;emphasis level="moderate"&gt;piquet&lt;/emphasis&gt;, le bois chaud. Tu vas tenir le fil. Il plante trop fort, et le bois penche. Pointe vers le bas, sans forcer. Le bois tape le sable, un toc. Il a tracé une ligne, comme un serpent. C'est le chemin. Maman glisse le tissu sous son autre bras. La ficelle pend contre sa manche. Piquet, je te porte. Le piquet est prêt, on avance.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir lève le &lt;emphasis level="moderate"&gt;piquet&lt;/emphasis&gt;, le bois chaud. Tu vas tenir le fil. Il plante trop fort, et le bois penche. Pointe vers le bas, sans forcer. Le bois tape le sable, un toc. Amir essuie le sable sur sa paume. Il a tracé une ligne, comme un serpent. C'est le chemin. Maman glisse le tissu sous son autre bras. La ficelle pend contre sa manche. Piquet, je te porte. Le piquet est prêt, on avance.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Amir lève le &lt;emphasis&gt;piquet&lt;/emphasis&gt;, le bois chaud. Tu vas tenir le fil. Il plante trop fort, et le bois penche. Pointe vers le bas, sans forcer. Le bois tape le sable, un toc. Il a tracé une ligne, comme un serpent. C'est le chemin. Maman glisse le tissu sous son autre bras. La ficelle pend contre sa manche. Piquet, je te porte. Le piquet est prêt, on avance. [pause]</t>
+          <t>Amir lève le &lt;emphasis&gt;piquet&lt;/emphasis&gt;, le bois chaud. Tu vas tenir le fil. Il plante trop fort, et le bois penche. Pointe vers le bas, sans forcer. Le bois tape le sable, un toc. Amir essuie le sable sur sa paume. Il a tracé une ligne, comme un serpent. C'est le chemin. Maman glisse le tissu sous son autre bras. La ficelle pend contre sa manche. Piquet, je te porte. Le piquet est prêt, on avance. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12125,6 +12135,7 @@
 narrateur|Il plante trop fort, et le bois penche.
 maman|Pointe vers le bas, sans forcer.
 narrateur|Le bois tape le sable, un toc.
+narrateur|Amir essuie le sable sur sa paume.
 papa|Il a tracé une ligne, comme un serpent.
 enfant-m|C'est le chemin.
 narrateur|Maman glisse le tissu sous son autre bras.
@@ -12730,17 +12741,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le bois du piquet est tiède. La crête de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le piquet penche, trop léger dans l'air. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Dans sa paume, le bois du piquet est tiède. La crête de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le piquet penche, trop léger dans l'air. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le bois du piquet est tiède. La &lt;emphasis level="moderate"&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le piquet penche, trop léger dans l'air. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le bois du piquet est tiède. La &lt;emphasis level="moderate"&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le piquet penche, trop léger dans l'air. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans sa paume, le bois du piquet est tiède. La &lt;emphasis&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le piquet penche, trop léger dans l'air. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans sa paume, le bois du piquet est tiède. La &lt;emphasis&gt;crête&lt;/emphasis&gt; de la dune souffle trop fort. Amir lance tout de suite, face au vent. Le piquet penche, trop léger dans l'air. Il va se déchirer ! La queue claque, trop prise. Le nez rouge se plie, minuscule. Amir souffle, les épaules basses. Ici, le vent est trop grand. Le rouge a besoin d'un vent plus petit. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -12885,6 +12896,7 @@
 enfant-m|Il va se déchirer !
 narrateur|La queue claque, trop prise.
 narrateur|Le nez rouge se plie, minuscule.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, le vent est trop grand.
 maman|Le rouge a besoin d'un vent plus petit.
 enfant-m|Alors on fait quoi ?
@@ -13116,17 +13128,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Il plante le piquet plus bas, loin de la crête. Amir descend, le bois contre le sable. L'air est plus petit, contre la pente. Il compte un, deux, le bois sans trembler. La pointe du piquet attend le sable. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, le bois tenait mieux.</t>
+          <t>Plus bas, d'abord. Il plante le piquet plus bas, loin de la crête. Amir descend, le bois contre le sable. L'air est plus petit, contre la pente. Il compte un, deux, le bois sans trembler. La pointe du piquet attend le sable. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, le bois tenait mieux.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Il plante le piquet plus bas, loin de la crête. Amir descend, le bois contre le sable. L'air est plus petit, contre la pente. Il compte un, deux, le bois sans trembler. La pointe du piquet attend le sable. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, le bois tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Il plante le piquet plus bas, loin de la crête. Amir descend, le bois contre le sable. L'air est plus petit, contre la pente. Il compte un, deux, le bois sans trembler. La pointe du piquet attend le sable. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, le bois tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Il plante le piquet plus bas, loin de la crête. Amir descend, le bois contre le sable. L'air est plus petit, contre la pente. Il compte un, deux, le bois sans trembler. La pointe du piquet attend le sable. Tu as regardé le vent. Ici, tu ne te déchires plus. Plus bas, le bois tenait mieux. [pause]</t>
+          <t>Plus bas, d'abord. Il plante le piquet plus bas, loin de la crête. Amir descend, le bois contre le sable. L'air est plus petit, contre la pente. Il compte un, deux, le bois sans trembler. La pointe du piquet attend le sable. Ici, le vent est plus petit. Ici, tu ne te déchires plus. Plus bas, le bois tenait mieux. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13266,7 +13278,7 @@
 narrateur|L'air est plus petit, contre la pente.
 narrateur|Il compte un, deux, le bois sans trembler.
 narrateur|La pointe du piquet attend le sable.
-papa|Tu as regardé le vent.
+papa|Ici, le vent est plus petit.
 enfant-m|Ici, tu ne te déchires plus.
 maman|Plus bas, le bois tenait mieux.</t>
         </is>
@@ -13481,17 +13493,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>On attend le vent. Il tient le piquet, sans le planter. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Planté, le piquet reste droit, sans bouger. Le vent s'est tu. Le rouge se lève, le bois sans penche. Le bois a eu son silence.</t>
+          <t>On attend le vent. Il tient le piquet, sans le planter. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Planté, le piquet reste droit, sans bouger. Le vent s'est tu. Le rouge se lève, le bois sans pencher. Le bois se tient, sans trembler.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend le vent. Il tient le piquet, sans le planter. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Planté, le piquet reste droit, sans bouger. Le vent s'est tu. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, le bois sans penche. Le bois a eu son silence.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend le vent. Il tient le piquet, sans le planter. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Planté, le piquet reste droit, sans bouger. Le vent s'est tu. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, le bois sans pencher. Le bois se tient, sans trembler.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>On attend le vent. Il tient le piquet, sans le planter. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Planté, le piquet reste droit, sans bouger. Le vent s'est tu. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, le bois sans penche. Le bois a eu son silence. [pause]</t>
+          <t>On attend le vent. Il tient le piquet, sans le planter. Le souffle passe, une fois, puis plus. Tu peux partir, maintenant. Planté, le piquet reste droit, sans bouger. Le vent s'est tu. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, le bois sans pencher. Le bois se tient, sans trembler. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13631,8 +13643,8 @@
 enfant-m|Tu peux partir, maintenant.
 narrateur|Planté, le piquet reste droit, sans bouger.
 papa|Le vent s'est tu.
-narrateur|Le rouge se lève, le bois sans penche.
-maman|Le bois a eu son silence.</t>
+narrateur|Le rouge se lève, le bois sans pencher.
+maman|Le bois se tient, sans trembler.</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr">
@@ -13664,17 +13676,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Quand le vent s'est tu, le bois est resté droit. On a compté, le bois sans penche. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. Le piquet garde un peu de sable, près du fil. Le bois reste droit, sans trembler.</t>
+          <t>Quand le vent s'est tu, le bois est resté droit. On a compté, le bois sans pencher. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. Le piquet garde un peu de sable, près du fil. Le bois reste droit, sans trembler.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le vent s'est tu, le bois est resté droit. On a compté, le bois sans penche. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. Le piquet garde un peu de sable, près du fil. Le bois reste droit, sans trembler.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le vent s'est tu, le bois est resté droit. On a compté, le bois sans pencher. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. Le piquet garde un peu de sable, près du fil. Le bois reste droit, sans trembler.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le vent s'est tu, le bois est resté droit. On a compté, le bois sans penche. Le silence a laissé partir le nez. Rentrez, le pin sent le chaud. Le piquet garde un peu de sable, près du fil. Le bois reste droit, sans trembler.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le vent s'est tu, le bois est resté droit. On a compté, le bois sans pencher. Le nez est parti, sans claquer. Rentrez, le pin sent le chaud. Le piquet garde un peu de sable, près du fil. Le bois reste droit, sans trembler.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13809,8 +13821,8 @@
       <c r="AW69" t="inlineStr">
         <is>
           <t>narrateur|Quand le vent s'est tu, le bois est resté droit.
-enfant-m|On a compté, le bois sans penche.
-papa|Le silence a laissé partir le nez.
+enfant-m|On a compté, le bois sans pencher.
+papa|Le nez est parti, sans claquer.
 maman|Rentrez, le pin sent le chaud.
 narrateur|Le piquet garde un peu de sable, près du fil.
 narrateur|Le bois reste droit, sans trembler.</t>
@@ -14209,17 +14221,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le bois du piquet est tiède. L'herbe de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Le piquet disparaît dans l'herbe, trop caché. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Dans sa paume, le bois du piquet est tiède. L'herbe de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Le piquet disparaît dans l'herbe, trop caché. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis level="moderate"&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Le piquet disparaît dans l'herbe, trop caché. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis level="moderate"&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Le piquet disparaît dans l'herbe, trop caché. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Le piquet disparaît dans l'herbe, trop caché. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis&gt;herbe&lt;/emphasis&gt; de la dune tient trop, trop verte. Amir court, et l'herbe attrape le fil. Le piquet disparaît dans l'herbe, trop caché. Le fil est coincé ! Une tige tire, puis une autre. Le rouge n'a plus d'air, trop bas. Amir souffle, les épaules basses. Ici, ça s'accroche trop. Le fil n'avance plus. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14364,6 +14376,7 @@
 enfant-m|Le fil est coincé !
 narrateur|Une tige tire, puis une autre.
 narrateur|Le rouge n'a plus d'air, trop bas.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, ça s'accroche trop.
 maman|Le fil n'avance plus.
 enfant-m|Alors on fait quoi ?
@@ -14595,17 +14608,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Plus court, d'abord. Il plante le piquet tout près, fil court. L'herbe n'atteint plus le fil. Le rouge se lève, tout petit. Planté, le piquet reste un instant, puis tient. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près.</t>
+          <t>Plus court, d'abord. Il plante le piquet tout près, fil court. L'herbe n'atteint plus le fil. Le rouge se lève, tout petit. Planté, le piquet reste un instant, puis tient. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus court, d'abord. Il plante le piquet tout près, fil court. L'herbe n'atteint plus le fil. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Planté, le piquet reste un instant, puis tient. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus court, d'abord. Il plante le piquet tout près, fil court. L'herbe n'atteint plus le fil. Le &lt;emphasis level="moderate"&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Planté, le piquet reste un instant, puis tient. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Plus court, d'abord. Il plante le piquet tout près, fil court. L'herbe n'atteint plus le fil. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Planté, le piquet reste un instant, puis tient. Le fil n'a plus accroché. Maintenant, tu me vois. Tu as commencé tout près. [pause]</t>
+          <t>Plus court, d'abord. Il plante le piquet tout près, fil court. L'herbe n'atteint plus le fil. Le &lt;emphasis&gt;rouge&lt;/emphasis&gt; se lève, tout petit. Planté, le piquet reste un instant, puis tient. Le fil n'a plus accroché. Maintenant, tu me vois. Le rouge est parti, tout près. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14746,7 +14759,7 @@
 narrateur|Planté, le piquet reste un instant, puis tient.
 maman|Le fil n'a plus accroché.
 enfant-m|Maintenant, tu me vois.
-papa|Tu as commencé tout près.</t>
+papa|Le rouge est parti, tout près.</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr">
@@ -14778,17 +14791,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la pointe du piquet, dans le sable nu. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. Le piquet garde un peu de sable, près du fil. La pointe du piquet, près, dans le sable nu.</t>
+          <t>Tout près, la pointe du piquet, dans le sable nu. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. Le piquet garde un peu de sable, près du fil. La pointe du piquet, près, dans le sable nu.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout près, la pointe du piquet, dans le sable nu. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. Le piquet garde un peu de sable, près du fil. La pointe du piquet, près, dans le sable nu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout près, la pointe du piquet, dans le sable nu. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. Le piquet garde un peu de sable, près du fil. La pointe du piquet, près, dans le sable nu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout près, la pointe du piquet, dans le sable nu. On a commencé tout court. Le silence vous a aidés. L'herbe sent le sel, moins fort. Le piquet garde un peu de sable, près du fil. La pointe du piquet, près, dans le sable nu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout près, la pointe du piquet, dans le sable nu. On a commencé tout court. Les tiges n'ont plus accroché. L'herbe sent le sel, moins fort. Le piquet garde un peu de sable, près du fil. La pointe du piquet, près, dans le sable nu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -14924,7 +14937,7 @@
         <is>
           <t>narrateur|Tout près, la pointe du piquet, dans le sable nu.
 enfant-m|On a commencé tout court.
-papa|Le silence vous a aidés.
+papa|Les tiges n'ont plus accroché.
 maman|L'herbe sent le sel, moins fort.
 narrateur|Le piquet garde un peu de sable, près du fil.
 narrateur|La pointe du piquet, près, dans le sable nu.</t>
@@ -14959,17 +14972,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>À genoux, on dénoue. À genoux, il dégage le piquet, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. La pointe du piquet attend le sable. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul.</t>
+          <t>À genoux, on dénoue. À genoux, il dégage le piquet, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. La pointe du piquet attend le sable. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;À genoux, on dénoue. À genoux, il dégage le piquet, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. La pointe du piquet attend le sable. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;À genoux, on dénoue. À genoux, il dégage le piquet, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. La pointe du piquet attend le sable. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>À genoux, on dénoue. À genoux, il dégage le piquet, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. La pointe du piquet attend le sable. Tu n'as pas tiré trop fort. C'est pour toi. Le nœud a lâché tout seul. [pause]</t>
+          <t>À genoux, on dénoue. À genoux, il dégage le piquet, sans tirer. Un nœud lâche, puis un autre. L'herbe se tait, plus loin, toute seule. La pointe du piquet attend le sable. Le nœud a lâché sans crier. C'est pour toi. Le nœud a lâché tout seul. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15108,7 +15121,7 @@
 narrateur|Un nœud lâche, puis un autre.
 narrateur|L'herbe se tait, plus loin, toute seule.
 narrateur|La pointe du piquet attend le sable.
-papa|Tu n'as pas tiré trop fort.
+papa|Le nœud a lâché sans crier.
 enfant-m|C'est pour toi.
 maman|Le nœud a lâché tout seul.</t>
         </is>
@@ -15142,17 +15155,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Quand le nœud s'est tu, un toc de bois, puis plus. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. Le piquet garde un peu de sable, près du fil. Un toc de bois, puis plus rien.</t>
+          <t>Quand le nœud s'est tu, un toc de bois, puis plus. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. Le piquet garde un peu de sable, près du fil. Un toc de bois, puis plus rien.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le nœud s'est tu, un toc de bois, puis plus. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. Le piquet garde un peu de sable, près du fil. Un toc de bois, puis plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Quand le nœud s'est tu, un toc de bois, puis plus. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. Le piquet garde un peu de sable, près du fil. Un toc de bois, puis plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le nœud s'est tu, un toc de bois, puis plus. On a dénoué, à genoux. Tu n'as pas tiré trop fort. Le fil a parlé tout seul. Le piquet garde un peu de sable, près du fil. Un toc de bois, puis plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Quand le nœud s'est tu, un toc de bois, puis plus. On a dénoué, à genoux. Le nœud a lâché sans crier. Le fil a parlé tout seul. Le piquet garde un peu de sable, près du fil. Un toc de bois, puis plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15288,7 +15301,7 @@
         <is>
           <t>narrateur|Quand le nœud s'est tu, un toc de bois, puis plus.
 enfant-m|On a dénoué, à genoux.
-papa|Tu n'as pas tiré trop fort.
+papa|Le nœud a lâché sans crier.
 maman|Le fil a parlé tout seul.
 narrateur|Le piquet garde un peu de sable, près du fil.
 narrateur|Un toc de bois, puis plus rien.</t>
@@ -15687,17 +15700,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le bois du piquet est tiède. L'écume lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le piquet s'enfonce, trop mou dans le sable. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?</t>
+          <t>Dans sa paume, le bois du piquet est tiède. L'écume lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le piquet s'enfonce, trop mou dans le sable. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis level="moderate"&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le piquet s'enfonce, trop mou dans le sable. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis level="moderate"&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le piquet s'enfonce, trop mou dans le sable. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le piquet s'enfonce, trop mou dans le sable. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Ici, ça mouille trop. Il lui faut du sec, et du temps. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans sa paume, le bois du piquet est tiède. L'&lt;emphasis&gt;écume&lt;/emphasis&gt; lèche le sable, trop près. Amir avance trop près, et une vague lèche. Le piquet s'enfonce, trop mou dans le sable. Il est tout mouillé ! Une vague revient, trop blanche. Le rouge n'a plus de vent, trop lourd. Amir souffle, les épaules basses. Ici, ça mouille trop. Le rouge est trop lourd, trop mouillé. Alors on fait quoi ? Tu vois comment, Amir ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15842,8 +15855,9 @@
 enfant-m|Il est tout mouillé !
 narrateur|Une vague revient, trop blanche.
 narrateur|Le rouge n'a plus de vent, trop lourd.
+narrateur|Amir souffle, les épaules basses.
 papa|Ici, ça mouille trop.
-maman|Il lui faut du sec, et du temps.
+maman|Le rouge est trop lourd, trop mouillé.
 enfant-m|Alors on fait quoi ?
 papa|Tu vois comment, Amir ?</t>
         </is>
@@ -16437,17 +16451,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>On attend la vague, d'abord. Il tient le piquet, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. La pointe du piquet attend le sable. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir.</t>
+          <t>On attend la vague, d'abord. Il tient le piquet, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. La pointe du piquet attend le sable. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend la vague, d'abord. Il tient le piquet, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. La pointe du piquet attend le sable. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend la vague, d'abord. Il tient le piquet, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. La pointe du piquet attend le sable. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>On attend la vague, d'abord. Il tient le piquet, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. La pointe du piquet attend le sable. Tu n'as pas couru dans l'eau. Tu es sec, maintenant. Tu as laissé la vague finir. [pause]</t>
+          <t>On attend la vague, d'abord. Il tient le piquet, puis regarde la vague. L'eau va, revient, puis se tait. Le sable redevient ferme, tout net. La pointe du piquet attend le sable. Tes pieds sont restés sur le sable. Tu es sec, maintenant. La vague a fini toute seule. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16586,9 +16600,9 @@
 narrateur|L'eau va, revient, puis se tait.
 narrateur|Le sable redevient ferme, tout net.
 narrateur|La pointe du piquet attend le sable.
-papa|Tu n'as pas couru dans l'eau.
+papa|Tes pieds sont restés sur le sable.
 enfant-m|Tu es sec, maintenant.
-maman|Tu as laissé la vague finir.</t>
+maman|La vague a fini toute seule.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr">
@@ -16620,17 +16634,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Après la vague, un trait de piquet, sec. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. Le piquet garde un peu de sable, près du fil. Un trait de piquet, sec, après la vague.</t>
+          <t>Après la vague, un trait de piquet, sec. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. Le piquet garde un peu de sable, près du fil. Un trait de piquet, sec, après la vague.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après la vague, un trait de piquet, sec. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. Le piquet garde un peu de sable, près du fil. Un trait de piquet, sec, après la vague.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après la vague, un trait de piquet, sec. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. Le piquet garde un peu de sable, près du fil. Un trait de piquet, sec, après la vague.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après la vague, un trait de piquet, sec. On a laissé l'eau se taire. Tu n'as pas couru dans l'eau. Tes doigts sentent le sel. Le piquet garde un peu de sable, près du fil. Un trait de piquet, sec, après la vague.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après la vague, un trait de piquet, sec. On a laissé l'eau se taire. Tes pieds sont restés sur le sable. Tes doigts sentent le sel. Le piquet garde un peu de sable, près du fil. Un trait de piquet, sec, après la vague.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16766,7 +16780,7 @@
         <is>
           <t>narrateur|Après la vague, un trait de piquet, sec.
 enfant-m|On a laissé l'eau se taire.
-papa|Tu n'as pas couru dans l'eau.
+papa|Tes pieds sont restés sur le sable.
 maman|Tes doigts sentent le sel.
 narrateur|Le piquet garde un peu de sable, près du fil.
 narrateur|Un trait de piquet, sec, après la vague.</t>
@@ -17159,7 +17173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17272,6 +17286,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>